<commit_message>
feat: cap nhat nhom hang vao menu mo rong san pham va dong bo du lieu mau phan cap
</commit_message>
<xml_diff>
--- a/backend/test_client/reports/Bảng kiểm thử Backend.xlsx
+++ b/backend/test_client/reports/Bảng kiểm thử Backend.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Test Cases" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -871,7 +871,7 @@
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>30/09/2026 13:17:25</t>
+          <t>06/10/2026 20:42:47</t>
         </is>
       </c>
     </row>

</xml_diff>